<commit_message>
chore(qa): execute performance and appium test suites and save reports
</commit_message>
<xml_diff>
--- a/automation/reports/excel/Automation_Test_Report.xlsx
+++ b/automation/reports/excel/Automation_Test_Report.xlsx
@@ -462,7 +462,7 @@
         <v>Passed</v>
       </c>
       <c r="F3">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -482,7 +482,7 @@
         <v>Passed</v>
       </c>
       <c r="F4">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -522,7 +522,7 @@
         <v>Passed</v>
       </c>
       <c r="F6">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -542,7 +542,7 @@
         <v>Passed</v>
       </c>
       <c r="F7">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -604,7 +604,7 @@
         <v>High</v>
       </c>
       <c r="E3">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -621,7 +621,7 @@
         <v>High</v>
       </c>
       <c r="E4">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -655,7 +655,7 @@
         <v>Medium</v>
       </c>
       <c r="E6">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -672,7 +672,7 @@
         <v>Medium</v>
       </c>
       <c r="E7">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>